<commit_message>
Fixed model changes and documentations
</commit_message>
<xml_diff>
--- a/Defect_Tracker Template_v0.1 InfySpringboard.xlsx
+++ b/Defect_Tracker Template_v0.1 InfySpringboard.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30431"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30516"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://infosystechnologies-my.sharepoint.com/personal/kamaljeet_kaur01_ad_infosys_com1/Documents/Infosys/CC/Events/Oct 2021 - Mar 2022/CC2.0/Internship/Jan-Apr 2022/Artifacts/internship/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:101_{A9B59A9A-789B-4A89-A90D-BB9A1B756E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF603EB2-F478-4C8E-A22F-A617BA1D0157}"/>
+  <xr:revisionPtr revIDLastSave="121" documentId="13_ncr:101_{A9B59A9A-789B-4A89-A90D-BB9A1B756E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55B9E6A7-444B-41E1-9E88-ADCAF95B1A5E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="35">
   <si>
     <t>Sl No</t>
   </si>
@@ -103,6 +103,33 @@
   </si>
   <si>
     <t>Added try/except blocks and ensured conn.close() is called on every transaction.</t>
+  </si>
+  <si>
+    <t>18/09/2026</t>
+  </si>
+  <si>
+    <t>Streamlit UI showing "0 Tool Calls" even when tools are executed.</t>
+  </si>
+  <si>
+    <t>Sprint 2</t>
+  </si>
+  <si>
+    <t>Updated investigation_agent.py to count m.type == "tool" from React agent messages and increment global_metrics.</t>
+  </si>
+  <si>
+    <t>Groq API throwing "Rate Limit Exceeded (429)" / "Request too large" errors.</t>
+  </si>
+  <si>
+    <t>Switched DEFAULT_MODEL to llama3-8b-8192</t>
+  </si>
+  <si>
+    <t>manage_incident tool crashing when provided an invalid action type.</t>
+  </si>
+  <si>
+    <t>Added validation to return an "Invalid action" error string</t>
+  </si>
+  <si>
+    <t>.</t>
   </si>
   <si>
     <t>User Interface</t>
@@ -121,7 +148,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="14">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -183,6 +210,28 @@
       <color rgb="FF1F2328"/>
       <name val="-Apple-System"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFD1D7E0"/>
+      <name val="-Apple-System"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="-Apple-System"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFD1D7E0"/>
+      <name val="Ui-Monospace"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Ui-Monospace"/>
     </font>
   </fonts>
   <fills count="3">
@@ -199,7 +248,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -222,11 +271,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -248,6 +306,12 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -558,11 +622,12 @@
     <col min="1" max="1" width="6.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.42578125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="42.140625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="43.7109375" style="4" customWidth="1"/>
     <col min="5" max="5" width="16" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="21.85546875" style="4" customWidth="1"/>
+    <col min="8" max="8" width="45.5703125" style="4" customWidth="1"/>
+    <col min="9" max="10" width="21.85546875" style="4" customWidth="1"/>
     <col min="11" max="11" width="16.85546875" style="4" customWidth="1"/>
     <col min="12" max="16384" width="17.5703125" style="4"/>
   </cols>
@@ -672,54 +737,120 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-    </row>
-    <row r="5" spans="1:11" ht="15.75">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.75">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
+    <row r="4" spans="1:11" ht="48.75">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="32.25">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="32.25">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="7" spans="1:11" ht="15.75">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
+      <c r="C7" s="12"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="6"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="3"/>
+      <c r="H7" s="14"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="6"/>
@@ -732,7 +863,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+      <c r="H8" s="13"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
@@ -745,7 +876,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="6"/>
       <c r="G9" s="5"/>
-      <c r="H9" s="3"/>
+      <c r="H9" s="11"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="6"/>
@@ -758,7 +889,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="6"/>
       <c r="G10" s="5"/>
-      <c r="H10" s="3"/>
+      <c r="H10" s="13"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="6"/>
@@ -771,7 +902,9 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
+      <c r="H11" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
@@ -925,22 +1058,22 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="7" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1082,6 +1215,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1090,20 +1229,14 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{191CB444-B9BF-4C91-94BD-600524521497}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}"/>
 </file>
</xml_diff>